<commit_message>
Master Sheet of all data created, still need to clean up duplicate taxon & site names
</commit_message>
<xml_diff>
--- a/Outputs/master_unique_lookups.xlsx
+++ b/Outputs/master_unique_lookups.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2659281f395c26b2/Documents/OCN682 Data Science Fundamentals in R/GroupA_AI_Data_Sprint/Outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_83CBFCB8217B2EB02AAF53AE94F737509B4A0CED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25E74E9D-EB9B-4876-ACCB-1BB2AA06EBB5}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_83479604C3E98B06971BF2AE94F737509B4A0229" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17181BDD-BA7C-4111-B181-AC186FC2A9E2}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Unique Sites Matrix" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="363">
   <si>
     <t>site_raw</t>
   </si>
@@ -578,6 +578,9 @@
     <t>dasya_spp</t>
   </si>
   <si>
+    <t>dendropoma_gregaria</t>
+  </si>
+  <si>
     <t>diadema_paucispinum</t>
   </si>
   <si>
@@ -689,6 +692,9 @@
     <t>halimeda_sp</t>
   </si>
   <si>
+    <t>haminoea_cymbalum</t>
+  </si>
+  <si>
     <t>haminoea_cymbalum_green_snail</t>
   </si>
   <si>
@@ -963,6 +969,9 @@
   </si>
   <si>
     <t>smaragdinella_calyculata</t>
+  </si>
+  <si>
+    <t>snail_dendropoma</t>
   </si>
   <si>
     <t>snail_dendropoma_gregarium</t>
@@ -1142,10 +1151,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1445,8 +1453,8 @@
   <dimension ref="A1:B55"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="25.6328125" customWidth="1"/>
+    <col min="1" max="1" width="25.36328125" customWidth="1"/>
+    <col min="2" max="2" width="27.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -1897,8 +1905,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A255"/>
+  <dimension ref="A1:A258"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="31.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1926,7 +1937,7 @@
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2301,7 +2312,7 @@
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+      <c r="A81" s="1" t="s">
         <v>185</v>
       </c>
     </row>
@@ -2311,7 +2322,7 @@
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A83" s="1" t="s">
+      <c r="A83" t="s">
         <v>187</v>
       </c>
     </row>
@@ -2321,12 +2332,12 @@
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+      <c r="A85" s="1" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A86" s="1" t="s">
+      <c r="A86" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2336,7 +2347,7 @@
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+      <c r="A88" s="1" t="s">
         <v>192</v>
       </c>
     </row>
@@ -2351,7 +2362,7 @@
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" s="1" t="s">
+      <c r="A91" t="s">
         <v>195</v>
       </c>
     </row>
@@ -2361,7 +2372,7 @@
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+      <c r="A93" s="1" t="s">
         <v>197</v>
       </c>
     </row>
@@ -2371,12 +2382,12 @@
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" s="1" t="s">
+      <c r="A95" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+      <c r="A96" s="1" t="s">
         <v>200</v>
       </c>
     </row>
@@ -2386,12 +2397,12 @@
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" s="1" t="s">
+      <c r="A98" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+      <c r="A99" s="1" t="s">
         <v>203</v>
       </c>
     </row>
@@ -2401,17 +2412,17 @@
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A101" s="1" t="s">
+      <c r="A101" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
+      <c r="A102" s="1" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A103" s="1" t="s">
+      <c r="A103" t="s">
         <v>207</v>
       </c>
     </row>
@@ -2421,17 +2432,17 @@
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
+      <c r="A105" s="1" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A106" s="1" t="s">
+      <c r="A106" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
+      <c r="A107" s="1" t="s">
         <v>211</v>
       </c>
     </row>
@@ -2446,7 +2457,7 @@
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A110" s="1" t="s">
+      <c r="A110" t="s">
         <v>214</v>
       </c>
     </row>
@@ -2456,7 +2467,7 @@
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
+      <c r="A112" s="1" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2501,12 +2512,12 @@
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A121" t="s">
+      <c r="A121" s="1" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A122" t="s">
+      <c r="A122" s="1" t="s">
         <v>226</v>
       </c>
     </row>
@@ -2556,12 +2567,12 @@
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A132" s="1" t="s">
+      <c r="A132" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A133" s="1" t="s">
+      <c r="A133" t="s">
         <v>237</v>
       </c>
     </row>
@@ -2571,12 +2582,12 @@
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A135" t="s">
+      <c r="A135" s="1" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A136" t="s">
+      <c r="A136" s="1" t="s">
         <v>240</v>
       </c>
     </row>
@@ -2591,12 +2602,12 @@
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A139" s="1" t="s">
+      <c r="A139" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A140" s="1" t="s">
+      <c r="A140" t="s">
         <v>244</v>
       </c>
     </row>
@@ -2611,27 +2622,27 @@
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A143" t="s">
+      <c r="A143" s="1" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A144" t="s">
+      <c r="A144" s="1" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A145" s="1" t="s">
+      <c r="A145" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A146" s="1" t="s">
+      <c r="A146" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A147" t="s">
+      <c r="A147" s="1" t="s">
         <v>251</v>
       </c>
     </row>
@@ -2641,17 +2652,17 @@
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A149" s="1" t="s">
+      <c r="A149" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A150" t="s">
+      <c r="A150" s="1" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A151" t="s">
+      <c r="A151" s="1" t="s">
         <v>255</v>
       </c>
     </row>
@@ -2661,7 +2672,7 @@
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A153" s="1" t="s">
+      <c r="A153" t="s">
         <v>257</v>
       </c>
     </row>
@@ -2681,7 +2692,7 @@
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A157" t="s">
+      <c r="A157" s="1" t="s">
         <v>261</v>
       </c>
     </row>
@@ -2746,12 +2757,12 @@
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A170" s="1" t="s">
+      <c r="A170" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A171" s="1" t="s">
+      <c r="A171" t="s">
         <v>275</v>
       </c>
     </row>
@@ -2761,12 +2772,12 @@
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A173" t="s">
+      <c r="A173" s="1" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A174" t="s">
+      <c r="A174" s="1" t="s">
         <v>278</v>
       </c>
     </row>
@@ -2791,22 +2802,22 @@
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A179" s="1" t="s">
+      <c r="A179" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A180" s="1" t="s">
+      <c r="A180" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A181" t="s">
+      <c r="A181" s="1" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A182" t="s">
+      <c r="A182" s="1" t="s">
         <v>286</v>
       </c>
     </row>
@@ -2826,22 +2837,22 @@
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A186" s="1" t="s">
+      <c r="A186" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A187" s="1" t="s">
+      <c r="A187" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A188" t="s">
+      <c r="A188" s="1" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A189" t="s">
+      <c r="A189" s="1" t="s">
         <v>293</v>
       </c>
     </row>
@@ -2856,17 +2867,17 @@
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A192" s="1" t="s">
+      <c r="A192" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A193" s="1" t="s">
+      <c r="A193" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A194" t="s">
+      <c r="A194" s="1" t="s">
         <v>298</v>
       </c>
     </row>
@@ -2881,12 +2892,12 @@
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A197" t="s">
+      <c r="A197" s="1" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A198" s="1" t="s">
+      <c r="A198" t="s">
         <v>302</v>
       </c>
     </row>
@@ -2896,7 +2907,7 @@
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A200" t="s">
+      <c r="A200" s="1" t="s">
         <v>304</v>
       </c>
     </row>
@@ -2921,22 +2932,22 @@
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A205" s="1" t="s">
+      <c r="A205" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A206" s="1" t="s">
+      <c r="A206" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A207" t="s">
+      <c r="A207" s="1" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A208" t="s">
+      <c r="A208" s="1" t="s">
         <v>312</v>
       </c>
     </row>
@@ -2956,12 +2967,12 @@
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A212" t="s">
+      <c r="A212" s="1" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A213" t="s">
+      <c r="A213" s="1" t="s">
         <v>317</v>
       </c>
     </row>
@@ -2976,12 +2987,12 @@
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A216" s="1" t="s">
+      <c r="A216" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A217" s="1" t="s">
+      <c r="A217" t="s">
         <v>321</v>
       </c>
     </row>
@@ -3006,22 +3017,22 @@
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A222" t="s">
+      <c r="A222" s="1" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A223" t="s">
+      <c r="A223" s="1" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A224" s="1" t="s">
+      <c r="A224" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A225" s="1" t="s">
+      <c r="A225" t="s">
         <v>329</v>
       </c>
     </row>
@@ -3046,12 +3057,12 @@
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A230" t="s">
+      <c r="A230" s="1" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A231" t="s">
+      <c r="A231" s="1" t="s">
         <v>335</v>
       </c>
     </row>
@@ -3061,17 +3072,17 @@
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A233" s="1" t="s">
+      <c r="A233" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A234" s="1" t="s">
+      <c r="A234" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A235" s="1" t="s">
+      <c r="A235" t="s">
         <v>339</v>
       </c>
     </row>
@@ -3081,12 +3092,12 @@
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A237" t="s">
+      <c r="A237" s="1" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A238" t="s">
+      <c r="A238" s="1" t="s">
         <v>342</v>
       </c>
     </row>
@@ -3096,7 +3107,7 @@
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A240" s="1" t="s">
+      <c r="A240" t="s">
         <v>344</v>
       </c>
     </row>
@@ -3111,7 +3122,7 @@
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A243" t="s">
+      <c r="A243" s="1" t="s">
         <v>347</v>
       </c>
     </row>
@@ -3121,7 +3132,7 @@
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A245" t="s">
+      <c r="A245" s="1" t="s">
         <v>349</v>
       </c>
     </row>
@@ -3131,7 +3142,7 @@
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A247" s="1" t="s">
+      <c r="A247" t="s">
         <v>351</v>
       </c>
     </row>
@@ -3141,17 +3152,17 @@
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A249" s="1" t="s">
+      <c r="A249" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A250" t="s">
+      <c r="A250" s="1" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A251" s="1" t="s">
+      <c r="A251" t="s">
         <v>355</v>
       </c>
     </row>
@@ -3166,13 +3177,28 @@
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A254" t="s">
+      <c r="A254" s="1" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A255" t="s">
+      <c r="A255" s="1" t="s">
         <v>359</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A256" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A257" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A258" t="s">
+        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
clean-ish master sheet, still need to add 2024-2026 metadata & fix duplicate site & taxon names
</commit_message>
<xml_diff>
--- a/Outputs/master_unique_lookups.xlsx
+++ b/Outputs/master_unique_lookups.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2659281f395c26b2/Documents/OCN682 Data Science Fundamentals in R/GroupA_AI_Data_Sprint/Outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_83479604C3E98B06971BF2AE94F737509B4A0229" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17181BDD-BA7C-4111-B181-AC186FC2A9E2}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_83479604C3E98B06971BF2AE94F737509B4A0229" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08C2AA3C-EA2F-49AC-9B1E-842F7F392230}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Unique Sites Matrix" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="365">
   <si>
     <t>site_raw</t>
   </si>
@@ -1110,6 +1110,12 @@
   </si>
   <si>
     <t>zoanthid_spp</t>
+  </si>
+  <si>
+    <t>unknown_bulbous_algae</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -1905,7 +1911,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A258"/>
+  <dimension ref="A1:B259"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.54296875" customWidth="1"/>
@@ -3111,93 +3117,101 @@
         <v>344</v>
       </c>
     </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A245" s="1" t="s">
+    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A245" t="s">
+        <v>363</v>
+      </c>
+      <c r="B245" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A246" s="1" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A246" t="s">
+    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A247" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A247" t="s">
+    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A248" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A248" t="s">
+    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A249" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A249" t="s">
+    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A250" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A250" s="1" t="s">
+    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A251" s="1" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A251" t="s">
+    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A252" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A252" s="1" t="s">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A253" s="1" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A253" t="s">
+    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A254" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A254" s="1" t="s">
+    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A255" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A255" s="1" t="s">
+    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A256" s="1" t="s">
         <v>359</v>
-      </c>
-    </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A256" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A259" t="s">
         <v>362</v>
       </c>
     </row>

</xml_diff>